<commit_message>
feat(quote): S9 quotes API with persisted lines, traces and logs (FN-17/18, TC-71)
- migration 0006: quote_headers (master version FK RESTRICT, inputs and
  metrics snapshot, amounts), quote_lines (calculated_* now, override_*
  reserved for FN-19), quote_traces, quote_validation_logs, audit
  triggers; cost_ratios.material_basis (NET | BBOX)
- POST /api/quotes from a DXF revision (2D metrics, title-block defaults
  for qty/material/thickness) or a document's 3D bodies, priced with the
  master data in force today; GET /api/quotes/{id} and
  /api/documents/{id}/quotes for estimators, reviewers, manufacturing
- master data: formulas validated on save (syntax + known names),
  material_basis in the bundle; G1 sheet 4 gains "재료 중량 기준"
- tests: trace completeness as a DB query, 3D quote, access rules

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011sSZvNfjmPHoXFa6o2Nfbi
</commit_message>
<xml_diff>
--- a/docs/inputs/G1_입력양식.xlsx
+++ b/docs/inputs/G1_입력양식.xlsx
@@ -1568,7 +1568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1732,6 +1732,24 @@
       <c r="D12" s="6" t="inlineStr">
         <is>
           <t>결과 금액이 달라지므로 꼭 선택</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>재료 중량 기준</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>순면적 / 소재 사각</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>판재: 순면적×두께 또는 외곽 사각×두께 (3D: 부피 / BBox)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master data: construction work items, adjust factors, price validity, QTO layers (Track 6-1)
Migration 0016 adds work_items (공종 단가: 재료·노무·경비, 손실률, 수량식) and
adjust_factors (지역·시점 보정) to the versioned bundle with the frozen/audit triggers,
valid_until on materials and price items, the indirect labour/cost rates of the
공사원가계산서, the QTO_LAYER mapping type and quote source CONSTRUCTION.
G1 gains optional sheets 9_공종단가 and 10_보정계수; older workbooks still import.
core/quote_engine/qto.py holds the QTO roles and measure names the work-item formulas
are validated against.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011sSZvNfjmPHoXFa6o2Nfbi
</commit_message>
<xml_diff>
--- a/docs/inputs/G1_입력양식.xlsx
+++ b/docs/inputs/G1_입력양식.xlsx
@@ -16,6 +16,8 @@
     <sheet name="6_표제란" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="7_샘플기대값" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="8_수기견적" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="9_공종단가" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10_보정계수" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -304,7 +306,7 @@
   <commentList>
     <comment ref="A4" authorId="0" shapeId="0">
       <text>
-        <t>외곽선(절단) / 절곡선 / 무시 / 표제란 / 펀칭 기준 직경(mm)</t>
+        <t>외곽선(절단) / 절곡선 / 무시 / 표제란 / 펀칭 기준 직경(mm). 공사 견적 수량산출: 실(면적) / 벽체 / 칸막이 / 문 / 창호 / 기구 / 덕트 / 배관 / 전선</t>
       </text>
     </comment>
     <comment ref="C4" authorId="0" shapeId="0">
@@ -390,6 +392,96 @@
     <comment ref="O4" authorId="0" shapeId="0">
       <text>
         <t>STEP만</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>AX-CAD</author>
+  </authors>
+  <commentList>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>영문·숫자·한글·.-_ (예: A-FLOOR)</t>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>건축 / 기계 / 전기 / 철거 등 내역서 분류</t>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>m2 / m / EA 등</t>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="0" shapeId="0">
+      <text>
+        <t>예: room_area_m2, wall_length_m * height_m, demo_wall_length_m * height_m, fixture_count. 접두어 new_ 신설 / demo_ 철거 / keep_ 유지</t>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="0" shapeId="0">
+      <text>
+        <t>할증률</t>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="0" shapeId="0">
+      <text>
+        <t>원/단위</t>
+      </text>
+    </comment>
+    <comment ref="I4" authorId="0" shapeId="0">
+      <text>
+        <t>원/단위</t>
+      </text>
+    </comment>
+    <comment ref="J4" authorId="0" shapeId="0">
+      <text>
+        <t>원/단위</t>
+      </text>
+    </comment>
+    <comment ref="K4" authorId="0" shapeId="0">
+      <text>
+        <t>YYYY-MM-DD. 지나면 견적 검증에서 경고</t>
+      </text>
+    </comment>
+    <comment ref="L4" authorId="0" shapeId="0">
+      <text>
+        <t>'예시'로 시작하는 행은 가져오지 않습니다</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>AX-CAD</author>
+  </authors>
+  <commentList>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>지역 / 시점</t>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>예: SEOUL, 2026Q4</t>
+      </text>
+    </comment>
+    <comment ref="C4" authorId="0" shapeId="0">
+      <text>
+        <t>0 초과 10 이하 (예: 1.05)</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>'예시'로 시작하는 행은 가져오지 않습니다</t>
       </text>
     </comment>
   </commentList>
@@ -685,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -798,43 +890,638 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>☐ 7_샘플기대값: 샘플 도면 DXF 15종 이상·STEP 5종 이상 + 사람이 잰 기대 메트릭</t>
+          <t>☐ (공사 견적 시) 9_공종단가·10_보정계수, 4_원가비율의 간접노무비율·간접공사비율</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>☐ 7_샘플기대값: 샘플 도면 DXF 15종 이상·STEP 5종 이상 + 사람이 잰 기대 메트릭</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>☐ 8_수기견적: 위 샘플 중 3건의 실제(수기) 견적서 금액 — 원 단위 일치 검증 기준(TC-67)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>사용처</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>1~6 시트 → 기준정보 화면 'G1 엑셀 가져오기'로 기준정보 초안에 반영(FN-16), 5·6은 2D 메트릭 규칙(FN-14).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>1~6·9·10 시트 → 기준정보 화면 'G1 엑셀 가져오기'로 기준정보 초안에 반영(FN-16), 5·6은 2D 메트릭 규칙(FN-14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>7·8 시트 → 메트릭·원가 계산 회귀 테스트 정답지(TC-60, TC-67). 가져오기 대상이 아닙니다.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>9_공종단가</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>공사·설비 견적 공종 단가. 수량은 도면 수량산출(실 면적·벽 길이·기구 수 등)에 수량식을 적용해 구합니다. 재료비 = 수량 × (1 + 손실률) × 재료단가, 노무비 = 수량 × 노무단가, 경비 = 수량 × 경비단가. 해당 없는 단가는 0. (선택 시트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>공종코드</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>공종</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>품명</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>규격</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>단위</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>수량식</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>손실률(%)</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>재료단가</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>노무단가</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>경비단가</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>유효기한</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>A-FLOOR</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>건축</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>바닥 타일</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>300×300</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>room_area_m2</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>A-PAINT</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>건축</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>벽체 도장</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>수성 2회</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>wall_length_m * height_m * 2</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>D-WALL</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>철거</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>벽체 철거</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>demo_wall_length_m * height_m</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>E-LIGHT</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>전기</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>등기구 설치</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>LED</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>fixture_count</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
+      <c r="L10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="7" t="n"/>
+      <c r="L11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="7" t="n"/>
+      <c r="L12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
+      <c r="L13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="n"/>
+      <c r="L14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
+      <c r="J15" s="7" t="n"/>
+      <c r="K15" s="7" t="n"/>
+      <c r="L15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+      <c r="J16" s="7" t="n"/>
+      <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n"/>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="7" t="n"/>
+      <c r="J17" s="7" t="n"/>
+      <c r="K17" s="7" t="n"/>
+      <c r="L17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:L2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>10_보정계수</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>단가 보정계수. 견적 작성 시 지역·시점을 고르면 모든 단가에 계수를 곱합니다(1 = 보정 없음). (선택 시트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>코드</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>계수</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>지역</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>SEOUL</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>시점</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>2026Q4</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1568,7 +2255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1688,66 +2375,102 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>절사 규칙</t>
+          <t>간접노무비율(%)</t>
         </is>
       </c>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>절사 / 반올림 / 올림</t>
+          <t>공사 견적만: 직접노무비 × 비율</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>금액 끝자리 처리</t>
+          <t>공사원가계산서</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>절사 단위(원)</t>
+          <t>간접공사비율(%)</t>
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>1 / 10 / 100 / 1000</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr"/>
+          <t>공사 견적만: (재료비 + 노무비) × 비율</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>기타경비·산재보험 등</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>절사 적용 시점</t>
+          <t>절사 규칙</t>
         </is>
       </c>
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>라인별 / 합계</t>
+          <t>절사 / 반올림 / 올림</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>결과 금액이 달라지므로 꼭 선택</t>
+          <t>금액 끝자리 처리</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>재료 중량 기준</t>
+          <t>절사 단위(원)</t>
         </is>
       </c>
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="6" t="inlineStr">
         <is>
+          <t>1 / 10 / 100 / 1000</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>절사 적용 시점</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>라인별 / 합계</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>결과 금액이 달라지므로 꼭 선택</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>재료 중량 기준</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
           <t>순면적 / 소재 사각</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>판재: 순면적×두께 또는 외곽 사각×두께 (3D: 부피 / BBox)</t>
         </is>

</xml_diff>

<commit_message>
P4-2: default machining rules (drill, tap, counterbore, countersink, milling, turning)
core/quote_engine/machining.py holds reference formulas (standard minutes
per piece, setup spread over the quantity) and prices. POST
/api/master-versions/{id}/machining-defaults adds them to a draft without
touching codes it already has; the master data page has a button for it,
and the G1 template shows them as example rows (regenerated).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011sSZvNfjmPHoXFa6o2Nfbi
</commit_message>
<xml_diff>
--- a/docs/inputs/G1_입력양식.xlsx
+++ b/docs/inputs/G1_입력양식.xlsx
@@ -246,7 +246,7 @@
     </comment>
     <comment ref="C4" authorId="0" shapeId="0">
       <text>
-        <t>다음 중 하나: cutting_length_mm, hole_count, punch_hole_count, bend_count, bend_length_mm, net_area_mm2, surface_area_mm2, volume_mm3, part_qty</t>
+        <t>다음 중 하나: cutting_length_mm, hole_count, punch_hole_count, bend_count, bend_length_mm, net_area_mm2, surface_area_mm2, volume_mm3, part_qty / 3D 가공: drill_length_mm, tap_count, tap_length_mm, counterbore_count, countersink_count, stock_volume_mm3, removed_volume_mm3, mill_removed_volume_mm3, turn_removed_volume_mm3, stock_diameter_mm, stock_length_mm</t>
       </text>
     </comment>
     <comment ref="D4" authorId="0" shapeId="0">
@@ -1780,7 +1780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1998,64 +1998,232 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>M-DRILL</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>드릴</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>hole_count</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>setup_min / part_qty + hole_count * index_min + drill_length_mm / feed_mm_per_min</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>setup_min=3, index_min=0.2, feed_mm_per_min=80</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>가공</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>예시: 3D 가공 참고값</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>M-TAP</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>탭</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>tap_count</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>tap_count * index_min + tap_length_mm * 2 / tap_mm_per_min</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>index_min=0.3, tap_mm_per_min=200</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>가공</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>예시: 3D 가공 참고값</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>M-CBORE</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>카운터보어</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>counterbore_count</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>counterbore_count * min_each</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>min_each=0.8</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>가공</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>예시: 3D 가공 참고값</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="7" t="n"/>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>M-CSINK</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>접시 가공</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>countersink_count</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>countersink_count * min_each</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>min_each=0.4</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>가공</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>예시: 3D 가공 참고값</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>M-MILL</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>밀링</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>mill_removed_volume_mm3</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>setup_min / part_qty + mill_removed_volume_mm3 / mrr_mm3_per_min</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>setup_min=30, mrr_mm3_per_min=12000</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>가공</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>예시: 3D 가공 참고값</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="7" t="n"/>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>M-TURN</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>선반</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>turn_removed_volume_mm3</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>setup_min / part_qty + turn_removed_volume_mm3 / mrr_mm3_per_min</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>setup_min=20, mrr_mm3_per_min=18000</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>가공</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>예시: 3D 가공 참고값</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -2096,6 +2264,66 @@
       <c r="F18" s="7" t="n"/>
       <c r="G18" s="7" t="n"/>
       <c r="H18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n"/>
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n"/>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n"/>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n"/>
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2255,7 +2483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2472,7 +2700,27 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>판재: 순면적×두께 또는 외곽 사각×두께 (3D: 부피 / BBox)</t>
+          <t>판재: 순면적×두께 또는 외곽 사각×두께 (3D: 부피 / 소재: 외곽+여유, 회전체는 환봉)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>소재 여유(mm)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>3D 소재: 면마다 더하는 가공 여유</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>각재 외곽·환봉 지름·길이</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
P4-5: purchased standard parts in the 3D BOM and quote
STANDARD feature (no body): KS hex bolt / socket bolt / nut / washer /
spring washer with size, length (bolts) and quantity per set. The model BOM
lists them under their item code (HB-M8x25 ...), a 3D quote prices them as
direct material at the PURCHASE price item with that code (traced to the
feature; a missing price is reported by validation). Migration 0021 adds the
feature and price types; G1 gets an optional 11_구매품단가 sheet. Model page:
규격품 dialog.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011sSZvNfjmPHoXFa6o2Nfbi
</commit_message>
<xml_diff>
--- a/docs/inputs/G1_입력양식.xlsx
+++ b/docs/inputs/G1_입력양식.xlsx
@@ -18,6 +18,7 @@
     <sheet name="8_수기견적" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="9_공종단가" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="10_보정계수" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11_구매품단가" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -480,6 +481,36 @@
       </text>
     </comment>
     <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>'예시'로 시작하는 행은 가져오지 않습니다</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>AX-CAD</author>
+  </authors>
+  <commentList>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>HB-M8x25(육각볼트), SB-M6x20(구멍붙이볼트), HN-M8(너트), PW-M8(평와셔), SW-M8(스프링와셔)</t>
+      </text>
+    </comment>
+    <comment ref="C4" authorId="0" shapeId="0">
+      <text>
+        <t>구매 단가</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>YYYY-MM-DD, 지나면 견적에 경고</t>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0">
       <text>
         <t>'예시'로 시작하는 행은 가져오지 않습니다</t>
       </text>
@@ -1525,6 +1556,180 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>11_구매품단가</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>규격품(볼트·너트·와셔) 구매 단가. 3D 모델의 규격품이 이 코드로 견적됩니다(직접재료비). (선택 시트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>품목코드</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>품명</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>단가(원/EA)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>유효기한</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>HB-M8x25</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>육각볼트 M8×25 (KS B 1002)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>HN-M8</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>육각너트 M8 (KS B 1012)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
P4-6a: standard construction costbook (표준품셈) in the master data
Migration 0022: costbook_items (with notice no., effective date, original
page, file SHA-256, extract method, reviewer), costbook_resources (labour /
material / equipment per unit), resource_prices (with price date and
source), work_items.costbook_item_code. Bundle validation ties them together;
activation needs a price for every resource a costbook-priced work item
uses. G1: sheets 12_품셈항목 / 13_품셈투입량 / 14_자원단가 with 15 example items
(2026 notice; numbers left to the original) and a trailing 품셈코드 column on
9_공종단가 (older workbooks still import). Master data page lists them.
Also restores the 5_레이어 row-error check lost in a test edit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011sSZvNfjmPHoXFa6o2Nfbi
</commit_message>
<xml_diff>
--- a/docs/inputs/G1_입력양식.xlsx
+++ b/docs/inputs/G1_입력양식.xlsx
@@ -19,6 +19,9 @@
     <sheet name="9_공종단가" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="10_보정계수" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="11_구매품단가" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12_품셈항목" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="13_품셈투입량" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="14_자원단가" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -234,6 +237,151 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>AX-CAD</author>
+  </authors>
+  <commentList>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>영문·숫자·.-_ (예: CB-PLASTER-W)</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>m2 / m3 / m / ton / 개소 등 (수량식 결과의 단위)</t>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>콘크리트 / 미장 / 도장 등</t>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="0" shapeId="0">
+      <text>
+        <t>예: 국토교통부 공고 제2025-1574호</t>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="0" shapeId="0">
+      <text>
+        <t>YYYY-MM-DD</t>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="0" shapeId="0">
+      <text>
+        <t>원문 PDF의 쪽 번호</t>
+      </text>
+    </comment>
+    <comment ref="I4" authorId="0" shapeId="0">
+      <text>
+        <t>원문 PDF 파일의 SHA-256(64자리 16진수, 선택)</t>
+      </text>
+    </comment>
+    <comment ref="J4" authorId="0" shapeId="0">
+      <text>
+        <t>수기 / PDF / OCR</t>
+      </text>
+    </comment>
+    <comment ref="L4" authorId="0" shapeId="0">
+      <text>
+        <t>YYYY-MM-DD</t>
+      </text>
+    </comment>
+    <comment ref="M4" authorId="0" shapeId="0">
+      <text>
+        <t>'예시'로 시작하는 행은 가져오지 않습니다</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>AX-CAD</author>
+  </authors>
+  <commentList>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>12_품셈항목의 코드</t>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>노무 / 재료 / 장비</t>
+      </text>
+    </comment>
+    <comment ref="C4" authorId="0" shapeId="0">
+      <text>
+        <t>14_자원단가의 코드 (예: L-PLASTERER)</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>품셈 단위 1당 (예: 미장공 0.06인/m2)</t>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>'예시'로 시작하는 행은 가져오지 않습니다</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment12.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>AX-CAD</author>
+  </authors>
+  <commentList>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>영문·숫자·.-_</t>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>노무 / 재료 / 장비</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>인 / kg / m3 / 시간 등</t>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>원/단위</t>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="0" shapeId="0">
+      <text>
+        <t>YYYY-MM-DD</t>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="0" shapeId="0">
+      <text>
+        <t>예: 대한건설협회 시중노임단가 2026 상반기</t>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="0" shapeId="0">
+      <text>
+        <t>YYYY-MM-DD, 지나면 견적에 경고</t>
+      </text>
+    </comment>
+    <comment ref="I4" authorId="0" shapeId="0">
+      <text>
+        <t>'예시'로 시작하는 행은 가져오지 않습니다</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -453,6 +601,11 @@
     <comment ref="L4" authorId="0" shapeId="0">
       <text>
         <t>'예시'로 시작하는 행은 가져오지 않습니다</t>
+      </text>
+    </comment>
+    <comment ref="M4" authorId="0" shapeId="0">
+      <text>
+        <t>12_품셈항목의 코드(선택). 넣으면 단가 칸은 비우고 품셈 투입량 × 14_자원단가로 계산</t>
       </text>
     </comment>
   </commentList>
@@ -974,7 +1127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -989,6 +1142,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1066,6 +1220,11 @@
           <t>비고</t>
         </is>
       </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>품셈코드</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1112,6 +1271,7 @@
           <t>예시</t>
         </is>
       </c>
+      <c r="M5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1158,6 +1318,7 @@
           <t>예시</t>
         </is>
       </c>
+      <c r="M6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -1200,6 +1361,7 @@
           <t>예시</t>
         </is>
       </c>
+      <c r="M7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -1246,20 +1408,56 @@
           <t>예시</t>
         </is>
       </c>
+      <c r="M8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>A-PLASTER</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>건축</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>벽 미장</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>시멘트 모르타르 18mm</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>wall_length_m * height_m * 2</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>예시: 표준품셈으로 단가 산출</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>CB-PLASTER-W</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -1274,6 +1472,7 @@
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
       <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -1288,6 +1487,7 @@
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
       <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -1302,6 +1502,7 @@
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -1316,6 +1517,7 @@
       <c r="J13" s="7" t="n"/>
       <c r="K13" s="7" t="n"/>
       <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1330,6 +1532,7 @@
       <c r="J14" s="7" t="n"/>
       <c r="K14" s="7" t="n"/>
       <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1344,6 +1547,7 @@
       <c r="J15" s="7" t="n"/>
       <c r="K15" s="7" t="n"/>
       <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -1358,6 +1562,7 @@
       <c r="J16" s="7" t="n"/>
       <c r="K16" s="7" t="n"/>
       <c r="L16" s="7" t="n"/>
+      <c r="M16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1372,6 +1577,7 @@
       <c r="J17" s="7" t="n"/>
       <c r="K17" s="7" t="n"/>
       <c r="L17" s="7" t="n"/>
+      <c r="M17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1386,10 +1592,26 @@
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
       <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A2:M2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -1724,6 +1946,1753 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>12_품셈항목</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>건설공사 표준품셈 항목(Track 8 P4-6). 수치는 2026년 적용 표준품셈 원문(CODIL·공공데이터포털 PDF)에서 옮기고 원문 페이지·검수자를 적습니다. 공종단가 시트의 '품셈코드'로 연결합니다. (선택 시트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>품셈코드</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>품명</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>규격</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>단위</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>분류</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>고시번호</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>적용일</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>원문 페이지</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>원문 SHA-256</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>추출방법</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>검수자</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>검수일</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>CB-CONC-PUMP</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>콘크리트 타설</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>펌프카, 철근콘크리트</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>콘크리트</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="6" t="n"/>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>CB-FORM-WALL</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>거푸집 설치·해체</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>합판, 벽</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>거푸집</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>CB-REBAR</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>철근 가공·조립</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>철근</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="n"/>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>CB-BRICK-1B</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>시멘트 벽돌 쌓기</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>1.0B</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>조적</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="6" t="n"/>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>CB-PLASTER-W</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>시멘트 모르타르 미장</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>벽, 18mm</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>미장</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="n"/>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>CB-PAINT-WB</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>수성페인트 칠</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>붓·롤러 2회</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>도장</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>CB-GYPSUM</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>석고보드 붙이기</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>1겹</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>수장</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>CB-CEIL-MBAR</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>경량철골 천장틀</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>M-BAR</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>수장</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>CB-TILE-FLOOR</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>바닥 타일 붙이기</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>압착</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>타일</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>CB-WATERPROOF</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>액체방수</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>2차</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>방수</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>CB-INSUL</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>단열재 설치</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>벽</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>단열</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>CB-DOOR-STEEL</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>강재 문틀 설치</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>외여닫이</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>개소</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>창호</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="6" t="n"/>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>CB-GLASS</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>유리 끼우기</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>복층 22mm</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>유리</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>CB-CONDUIT</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>전선관 배관</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>PVC 16C</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>전기</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="n"/>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>CB-PIPE-25A</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>강관 배관</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>25A</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>기계설비</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>국토교통부 공고 제2025-1574호</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>수기</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n"/>
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="7" t="n"/>
+      <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="7" t="n"/>
+      <c r="K21" s="7" t="n"/>
+      <c r="L21" s="7" t="n"/>
+      <c r="M21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n"/>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="7" t="n"/>
+      <c r="K22" s="7" t="n"/>
+      <c r="L22" s="7" t="n"/>
+      <c r="M22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n"/>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="7" t="n"/>
+      <c r="K23" s="7" t="n"/>
+      <c r="L23" s="7" t="n"/>
+      <c r="M23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n"/>
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="7" t="n"/>
+      <c r="I24" s="7" t="n"/>
+      <c r="J24" s="7" t="n"/>
+      <c r="K24" s="7" t="n"/>
+      <c r="L24" s="7" t="n"/>
+      <c r="M24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n"/>
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="7" t="n"/>
+      <c r="K25" s="7" t="n"/>
+      <c r="L25" s="7" t="n"/>
+      <c r="M25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n"/>
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="7" t="n"/>
+      <c r="J26" s="7" t="n"/>
+      <c r="K26" s="7" t="n"/>
+      <c r="L26" s="7" t="n"/>
+      <c r="M26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="n"/>
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="n"/>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="7" t="n"/>
+      <c r="J27" s="7" t="n"/>
+      <c r="K27" s="7" t="n"/>
+      <c r="L27" s="7" t="n"/>
+      <c r="M27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n"/>
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+      <c r="H28" s="7" t="n"/>
+      <c r="I28" s="7" t="n"/>
+      <c r="J28" s="7" t="n"/>
+      <c r="K28" s="7" t="n"/>
+      <c r="L28" s="7" t="n"/>
+      <c r="M28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="n"/>
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="7" t="n"/>
+      <c r="J29" s="7" t="n"/>
+      <c r="K29" s="7" t="n"/>
+      <c r="L29" s="7" t="n"/>
+      <c r="M29" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:M2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>13_품셈투입량</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>품셈 항목 단위당 투입량: 노무(직종별 인), 재료(자재 수량), 장비(시간). 공사비 = 수량 × Σ(투입량 × 자원단가). (선택 시트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>품셈코드</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>자원구분</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>자원코드</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>단위당 투입량</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>CB-PLASTER-W</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>노무</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>L-PLASTERER</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>CB-PLASTER-W</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>노무</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>L-WORKER</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>CB-PLASTER-W</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>재료</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>M-CEMENT</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>CB-PLASTER-W</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>재료</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>M-SAND</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>CB-CONC-PUMP</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>장비</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>E-PUMPCAR</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n"/>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>14_자원단가</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>자원 단가: 노임(원/인, 시중노임단가), 자재(원/단위), 기계경비(원/시간, 건설기계 기계경비 산출표). 기준일·출처를 적습니다. (선택 시트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>자원코드</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>자원구분</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>자원명</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>단위</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>단가</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>기준일</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>유효기한</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>L-PLASTERER</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>노무</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>미장공</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>인</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>대한건설협회 시중노임단가</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>L-WORKER</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>노무</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>보통인부</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>인</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>대한건설협회 시중노임단가</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>M-CEMENT</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>재료</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>시멘트</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>M-SAND</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>재료</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>모래</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>E-PUMPCAR</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>장비</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>콘크리트 펌프카</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>시간</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>건설기계 기계경비 산출표</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n"/>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
P4-6c: drawing objects (layer/block, attribute, length/area/volume/count, factor, waste) as obj_<code> QTO measures
Master data qto_objects (migration 0022, G1 sheet 15_도면객체, master page table);
work item formulas may read obj_<code> with new_/demo_/keep_ prefixes; quote lines trace
to the objects' entity handles.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011sSZvNfjmPHoXFa6o2Nfbi
</commit_message>
<xml_diff>
--- a/docs/inputs/G1_입력양식.xlsx
+++ b/docs/inputs/G1_입력양식.xlsx
@@ -22,6 +22,7 @@
     <sheet name="12_품셈항목" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="13_품셈투입량" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="14_자원단가" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="15_도면객체" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -371,6 +372,56 @@
     <comment ref="H4" authorId="0" shapeId="0">
       <text>
         <t>YYYY-MM-DD, 지나면 견적에 경고</t>
+      </text>
+    </comment>
+    <comment ref="I4" authorId="0" shapeId="0">
+      <text>
+        <t>'예시'로 시작하는 행은 가져오지 않습니다</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment13.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>AX-CAD</author>
+  </authors>
+  <commentList>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>영문 소문자·숫자·_ (예: slab). 수량식 이름 = obj_코드</t>
+      </text>
+    </comment>
+    <comment ref="C4" authorId="0" shapeId="0">
+      <text>
+        <t>예: A-SLAB*, 슬래브* (비우면 모든 레이어)</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>예: COL-*, 기둥* (블록만 셀 때)</t>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>블록 속성 값(숫자)을 수량으로 쓸 때 태그 (예: QTY, VOL)</t>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="0" shapeId="0">
+      <text>
+        <t>길이(m) / 면적(m2) / 체적 / 개수</t>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="0" shapeId="0">
+      <text>
+        <t>곱하는 값. 체적은 두께(m), 단위 환산 등 (기본 1)</t>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="0" shapeId="0">
+      <text>
+        <t>할증·손실 (예: 5)</t>
       </text>
     </comment>
     <comment ref="I4" authorId="0" shapeId="0">
@@ -3699,6 +3750,309 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>15_도면객체</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>도면 객체 → 수량: 레이어·블록 이름(쉼표로 여러 개, * 와일드카드)에 맞는 객체를 길이·면적·체적·개수로 재고, 환산계수 × (1 + 할증률)을 곱해 9_공종단가 수량식에서 obj_코드 로 씁니다 (new_/demo_/keep_obj_코드 도 가능). (선택 시트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>코드</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>레이어</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>블록</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>속성 태그</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>수량유형</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>환산계수</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>할증률(%)</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>slab</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>슬래브 콘크리트</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>A-SLAB*</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>체적</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>기둥</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>COL-*</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>개수</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>tray</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>케이블 트레이</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>E-TRAY*</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>길이</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n"/>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>